<commit_message>
más cambios y correcciones
</commit_message>
<xml_diff>
--- a/exceldoc/ESTRATEGIA DE REQUISITOS - METAFIT.xlsx
+++ b/exceldoc/ESTRATEGIA DE REQUISITOS - METAFIT.xlsx
@@ -16,7 +16,7 @@
     <numFmt numFmtId="164" formatCode="d/M/yyyy"/>
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Aptos Narrow"/>
       <color theme="1"/>
@@ -45,6 +45,9 @@
       <name val="Aptos Narrow"/>
       <color theme="1"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="5">
@@ -295,7 +298,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -420,6 +423,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -696,7 +705,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA1000"/>
+  <dimension ref="A1:AB1000"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="20.13" customWidth="1" style="40" min="1" max="1"/>
@@ -816,6 +825,11 @@
       <c r="Y1" s="42" t="n"/>
       <c r="Z1" s="42" t="n"/>
       <c r="AA1" s="43" t="n"/>
+      <c r="AB1" s="51" t="inlineStr">
+        <is>
+          <t>CRITERIOS DE ACEPTACIÓN</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="44" t="n"/>
@@ -941,6 +955,14 @@
       <c r="Y3" s="21" t="n"/>
       <c r="Z3" s="21" t="n"/>
       <c r="AA3" s="21" t="n"/>
+      <c r="AB3" s="52" t="inlineStr">
+        <is>
+          <t>1. Se muestra el formulario de inicio de sesión (correo y contraseña).
+2. Con credenciales válidas se accede a la app (Home).
+3. Con credenciales inválidas se muestra un mensaje de error claro y no se accede.
+4. La sesión queda persistida al cerrar y reabrir la app.</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="63" customHeight="1" s="40">
       <c r="A4" s="48" t="n"/>
@@ -1000,6 +1022,14 @@
       <c r="Y4" s="20" t="n"/>
       <c r="Z4" s="20" t="n"/>
       <c r="AA4" s="21" t="n"/>
+      <c r="AB4" s="52" t="inlineStr">
+        <is>
+          <t>1. Existe una opción de cerrar sesión accesible desde el menú.
+2. Al confirmar, se limpian token y datos de sesión almacenados.
+3. Tras cerrar sesión se redirige a la pantalla de Login.
+4. No es posible acceder a pantallas privadas sin estar autenticado.</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="78.75" customHeight="1" s="40">
       <c r="A5" s="48" t="n"/>
@@ -1894,6 +1924,14 @@
       <c r="Y19" s="21" t="n"/>
       <c r="Z19" s="21" t="n"/>
       <c r="AA19" s="21" t="n"/>
+      <c r="AB19" s="52" t="inlineStr">
+        <is>
+          <t>1. El afiliado ve sus datos personales (nombres, apellidos, correo, teléfono, edad).
+2. Se muestran peso, altura e IMC reales desde la base de datos.
+3. Se puede editar peso, altura, teléfono y correo desde la pantalla Perfil.
+4. Los cambios se guardan y reflejan al recargar la pantalla.</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="78.75" customHeight="1" s="40">
       <c r="A20" s="48" t="n"/>
@@ -2134,6 +2172,13 @@
       <c r="Y23" s="21" t="n"/>
       <c r="Z23" s="21" t="n"/>
       <c r="AA23" s="21" t="n"/>
+      <c r="AB23" s="52" t="inlineStr">
+        <is>
+          <t>1. El afiliado ve sus restricciones médicas (nombre, tipo y efecto relevante).
+2. Las restricciones se muestran como badges/píldoras claros.
+3. Se indica un mensaje o descripción del efecto de cada restricción.</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="110.25" customHeight="1" s="40">
       <c r="A24" s="49" t="n"/>
@@ -2383,6 +2428,14 @@
       <c r="Y27" s="21" t="n"/>
       <c r="Z27" s="21" t="n"/>
       <c r="AA27" s="21" t="n"/>
+      <c r="AB27" s="52" t="inlineStr">
+        <is>
+          <t>1. El afiliado ve la lista de sus ciclos de entrenamiento.
+2. Cada ciclo muestra número, objetivo físico, fechas y días de disponibilidad.
+3. Se indica cuál es el ciclo activo.
+4. Se muestra un resumen del historial de ciclos.</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="63" customHeight="1" s="40">
       <c r="A28" s="48" t="n"/>
@@ -3158,6 +3211,14 @@
       <c r="Y40" s="37" t="n"/>
       <c r="Z40" s="37" t="n"/>
       <c r="AA40" s="37" t="n"/>
+      <c r="AB40" s="52" t="inlineStr">
+        <is>
+          <t>1. El afiliado ve la rutina del día con sus ejercicios.
+2. Los ejercicios mostrados corresponden al grupo muscular del día (coherentes con el plan).
+3. Se muestra grupo muscular, series, repeticiones, peso y descanso de cada ejercicio.
+4. Se puede seleccionar otro día de la semana y ver su rutina.</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="63" customHeight="1" s="40">
       <c r="A41" s="46" t="inlineStr">
@@ -3761,6 +3822,14 @@
       <c r="Y50" s="37" t="n"/>
       <c r="Z50" s="37" t="n"/>
       <c r="AA50" s="37" t="n"/>
+      <c r="AB50" s="52" t="inlineStr">
+        <is>
+          <t>1. El afiliado ve su plan nutricional diario.
+2. Las comidas se organizan por horario (Desayuno, Almuerzo, Cena, Snack).
+3. Cada comida muestra sus alimentos con macros (calorías, proteínas, carbos, grasas).
+4. Se muestra la meta de agua diaria (2L / 8 vasos) con barra de progreso.</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="126" customHeight="1" s="40">
       <c r="A51" s="46" t="inlineStr">
@@ -4377,6 +4446,15 @@
       <c r="Y60" s="37" t="n"/>
       <c r="Z60" s="37" t="n"/>
       <c r="AA60" s="37" t="n"/>
+      <c r="AB60" s="52" t="inlineStr">
+        <is>
+          <t>1. El afiliado ve su historial de progreso físico (peso, IMC, grasa, músculo).
+2. Se muestra un gráfico de evolución de peso a lo largo del tiempo.
+3. Se muestra un gráfico de volumen levantado por semana.
+4. Se muestra un gráfico de cumplimiento nutricional (dona).
+5. Las fechas se muestran en formato DD/MM/YYYY.</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="63" customHeight="1" s="40">
       <c r="A61" s="48" t="n"/>
@@ -4440,6 +4518,15 @@
       <c r="Y61" s="37" t="n"/>
       <c r="Z61" s="37" t="n"/>
       <c r="AA61" s="37" t="n"/>
+      <c r="AB61" s="52" t="inlineStr">
+        <is>
+          <t>1. El afiliado puede marcar ejercicios de su rutina como completados.
+2. Puede registrar peso REAL usado (kg).
+3. Puede registrar repeticiones REALES realizadas.
+4. Puede registrar series REALES realizadas.
+5. El sistema calcula el volumen total (peso × reps × series).</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="47.25" customHeight="1" s="40">
       <c r="A62" s="48" t="n"/>
@@ -4503,6 +4590,13 @@
       <c r="Y62" s="37" t="n"/>
       <c r="Z62" s="37" t="n"/>
       <c r="AA62" s="37" t="n"/>
+      <c r="AB62" s="52" t="inlineStr">
+        <is>
+          <t>1. El afiliado consulta los ejercicios completados de su rutina.
+2. Se muestra fecha, ejercicio, series×reps, peso usado y volumen.
+3. Los registros se muestran ordenados y con fechas legibles (DD/MM/YYYY).</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="47.25" customHeight="1" s="40">
       <c r="A63" s="48" t="n"/>
@@ -4566,6 +4660,13 @@
       <c r="Y63" s="37" t="n"/>
       <c r="Z63" s="37" t="n"/>
       <c r="AA63" s="37" t="n"/>
+      <c r="AB63" s="52" t="inlineStr">
+        <is>
+          <t>1. El afiliado registra vasos de agua consumidos en el día.
+2. Se muestra la meta diaria 2L (8 vasos) con una barra de progreso.
+3. El progreso se guarda y persiste al recargar.</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="47.25" customHeight="1" s="40">
       <c r="A64" s="48" t="n"/>
@@ -4629,6 +4730,13 @@
       <c r="Y64" s="37" t="n"/>
       <c r="Z64" s="37" t="n"/>
       <c r="AA64" s="37" t="n"/>
+      <c r="AB64" s="52" t="inlineStr">
+        <is>
+          <t>1. El afiliado consulta los vasos de agua registrados.
+2. Se muestra el historial con fecha y cantidad (x/8).
+3. Se indica si se cumplió la meta del día.</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="141.75" customHeight="1" s="40">
       <c r="A65" s="49" t="n"/>
@@ -4692,6 +4800,15 @@
       <c r="Y65" s="37" t="n"/>
       <c r="Z65" s="37" t="n"/>
       <c r="AA65" s="37" t="n"/>
+      <c r="AB65" s="52" t="inlineStr">
+        <is>
+          <t>1. El afiliado puede registrar alimentos consumidos por comida (horario).
+2. Puede registrar la cantidad REAL consumida en gramos.
+3. El sistema calcula automáticamente las calorías consumidas.
+4. El sistema calcula proteínas, carbohidratos y grasas consumidas.
+5. Los nutrientes se muestran al consumir y quedan guardados.</t>
+        </is>
+      </c>
     </row>
     <row r="66" ht="15.75" customHeight="1" s="40">
       <c r="A66" s="38" t="inlineStr">
@@ -4763,6 +4880,14 @@
       <c r="Y66" s="37" t="n"/>
       <c r="Z66" s="37" t="n"/>
       <c r="AA66" s="37" t="n"/>
+      <c r="AB66" s="52" t="inlineStr">
+        <is>
+          <t>1. El afiliado solicita un enlace de recuperación de contraseña.
+2. Se envía un enlace/token de recuperación.
+3. El afiliado puede restablecer su contraseña con el token.
+4. Con la nueva contraseña puede iniciar sesión.</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="15.75" customHeight="1" s="40">
       <c r="A67" s="38" t="n"/>
@@ -4826,6 +4951,14 @@
       <c r="Y67" s="37" t="n"/>
       <c r="Z67" s="37" t="n"/>
       <c r="AA67" s="37" t="n"/>
+      <c r="AB67" s="52" t="inlineStr">
+        <is>
+          <t>1. El afiliado puede subir una foto de perfil desde la app.
+2. La foto se puede tomar con la cámara o seleccionar de la galería.
+3. La nueva foto se muestra en el perfil y se conserva al recargar.
+4. La foto se sube al backend (Cloudinary o local).</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="15.75" customHeight="1" s="40">
       <c r="A68" s="38" t="inlineStr">
@@ -4893,6 +5026,13 @@
       <c r="Y68" s="37" t="n"/>
       <c r="Z68" s="37" t="n"/>
       <c r="AA68" s="37" t="n"/>
+      <c r="AB68" s="52" t="inlineStr">
+        <is>
+          <t>1. La app permite cambiar entre tema claro y oscuro.
+2. La preferencia de tema queda persistida entre sesiones.
+3. La selección de tema se aplica a todas las pantallas.</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="15.75" customHeight="1" s="40">
       <c r="A69" s="38" t="n"/>
@@ -4952,6 +5092,14 @@
       <c r="Y69" s="37" t="n"/>
       <c r="Z69" s="37" t="n"/>
       <c r="AA69" s="37" t="n"/>
+      <c r="AB69" s="52" t="inlineStr">
+        <is>
+          <t>1. La app solicita permiso de notificaciones push.
+2. Se reciben notificaciones push relevantes (recordatorios, avisos).
+3. Se maneja correctamente el token de push del dispositivo.
+4. Al tocar la notificación se abre la pantalla correspondiente.</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="15.75" customHeight="1" s="40">
       <c r="A70" s="38" t="n"/>

</xml_diff>